<commit_message>
feat: Chronicle Points primitive — 20% of dated base rate on Chronicle Farm USDS, Grove only; Sky-funded in sky_total (#166)
Co-authored-by: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/settlements/grove/2026-07/grove_settlement_july_2026.xlsx
+++ b/settlements/grove/2026-07/grove_settlement_july_2026.xlsx
@@ -458,7 +458,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B27"/>
+  <dimension ref="A1:B28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="1" max="1"/>
@@ -515,168 +515,178 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr"/>
-      <c r="B7" s="4" t="n">
-        <v>3473819.385647459</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>+ chronicle_points (20% of base rate on Chronicle Farm USDS)</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>13102.07817737222</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr"/>
+      <c r="B8" s="4" t="n">
+        <v>3486921.463824832</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
         <is>
           <t>Sky side</t>
         </is>
       </c>
-      <c r="B9" s="2" t="inlineStr">
+      <c r="B10" s="2" t="inlineStr">
         <is>
           <t>USD</t>
         </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>CoF on utilized (BR × Net_Subs)</t>
-        </is>
-      </c>
-      <c r="B10" s="3" t="n">
-        <v>3299017.138218012</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
+          <t>CoF on utilized (BR × Net_Subs)</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>3299017.138218012</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
           <t>+ SDE revenue (Sky-Direct, full to Sky)</t>
         </is>
       </c>
-      <c r="B11" s="3" t="n">
+      <c r="B12" s="3" t="n">
         <v>4704533.195761743</v>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" t="inlineStr"/>
-      <c r="B12" s="4" t="n">
+    <row r="13">
+      <c r="A13" t="inlineStr"/>
+      <c r="B13" s="4" t="n">
         <v>8003550.333979755</v>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="2" t="inlineStr">
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
         <is>
           <t>Sky Revenue (max) — BR × full ilk debt, no deductions</t>
         </is>
       </c>
-      <c r="B14" s="2" t="inlineStr">
+      <c r="B15" s="2" t="inlineStr">
         <is>
           <t>USD</t>
         </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>CoF on Net_Subs (actual BR × utilized)</t>
-        </is>
-      </c>
-      <c r="B15" s="3" t="n">
-        <v>3299017.138218012</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
+          <t>CoF on Net_Subs (actual BR × utilized)</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n">
+        <v>3299017.138218012</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
           <t>reduction from idle/SDE deductions</t>
         </is>
       </c>
-      <c r="B16" s="3" t="n">
+      <c r="B17" s="3" t="n">
         <v>-5044716.385903903</v>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" t="inlineStr"/>
-      <c r="B17" s="4" t="n">
+    <row r="18">
+      <c r="A18" t="inlineStr"/>
+      <c r="B18" s="4" t="n">
         <v>8343733.524121915</v>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="2" t="inlineStr">
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
         <is>
           <t>Comparison (Grove-style "Profit to Grove")</t>
         </is>
       </c>
-      <c r="B19" s="2" t="inlineStr">
+      <c r="B20" s="2" t="inlineStr">
         <is>
           <t>USD</t>
         </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>prime_agent_revenue</t>
-        </is>
-      </c>
-      <c r="B20" s="3" t="n">
-        <v>3372897.374026904</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
+          <t>prime_agent_revenue</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="n">
+        <v>3372897.374026904</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
           <t>− CoF (deducted per-venue in display)</t>
         </is>
       </c>
-      <c r="B21" s="3" t="n">
+      <c r="B22" s="3" t="n">
         <v>-3299017.138218012</v>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" t="inlineStr"/>
-      <c r="B22" s="4" t="n">
+    <row r="23">
+      <c r="A23" t="inlineStr"/>
+      <c r="B23" s="4" t="n">
         <v>73880.23580889196</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>Period</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>2026-07-01 → 2026-07-31 (31 days)</t>
-        </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Pin blocks</t>
+          <t>Period</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>avalanche_c=91716609, base=49376526, ethereum=25656292, monad=92053501, plume=84574746</t>
+          <t>2026-07-01 → 2026-07-31 (31 days)</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Generated</t>
+          <t>Pin blocks</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>2026-08-03T23:48:56+00:00</t>
+          <t>avalanche_c=91716609, base=49376526, ethereum=25656292, monad=92053501, plume=84574746</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
+          <t>Generated</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>2026-08-04T23:14:13+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
           <t>Pipeline</t>
         </is>
       </c>
-      <c r="B27" t="inlineStr">
+      <c r="B28" t="inlineStr">
         <is>
           <t>0.1.0</t>
         </is>

</xml_diff>

<commit_message>
fix(grove): capture direct-aToken Merkl payouts — Jul 2026 E1 +$1.47M (#169)
Co-authored-by: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/settlements/grove/2026-07/grove_settlement_july_2026.xlsx
+++ b/settlements/grove/2026-07/grove_settlement_july_2026.xlsx
@@ -491,7 +491,7 @@
         </is>
       </c>
       <c r="B4" s="3" t="n">
-        <v>3372897.374026904</v>
+        <v>4841078.809624951</v>
       </c>
     </row>
     <row r="5">
@@ -527,7 +527,7 @@
     <row r="8">
       <c r="A8" t="inlineStr"/>
       <c r="B8" s="4" t="n">
-        <v>3486921.463824832</v>
+        <v>4955102.899422878</v>
       </c>
     </row>
     <row r="10">
@@ -625,7 +625,7 @@
         </is>
       </c>
       <c r="B21" s="3" t="n">
-        <v>3372897.374026904</v>
+        <v>4841078.809624951</v>
       </c>
     </row>
     <row r="22">
@@ -641,7 +641,7 @@
     <row r="23">
       <c r="A23" t="inlineStr"/>
       <c r="B23" s="4" t="n">
-        <v>73880.23580889196</v>
+        <v>1542061.671406939</v>
       </c>
     </row>
     <row r="25">
@@ -676,7 +676,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2026-08-04T23:14:13+00:00</t>
+          <t>2026-08-05T22:21:57+00:00</t>
         </is>
       </c>
     </row>
@@ -1256,10 +1256,10 @@
         <v>117961.8010746321</v>
       </c>
       <c r="I8" s="5" t="n">
-        <v>0</v>
+        <v>1468181.435598047</v>
       </c>
       <c r="J8" s="5" t="n">
-        <v>117961.8010746321</v>
+        <v>1586143.236672679</v>
       </c>
       <c r="K8" s="5" t="n">
         <v>0</v>
@@ -1277,7 +1277,7 @@
         <v>227935.6692296159</v>
       </c>
       <c r="P8" s="5" t="n">
-        <v>-109973.8681549838</v>
+        <v>1358207.567443063</v>
       </c>
       <c r="Q8" s="5" t="n">
         <v>0</v>

</xml_diff>